<commit_message>
docs: update CHANGES_LOG.txt and changes.txt with GitHub push and Vercel production deployment records
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -991,7 +991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4485,6 +4485,162 @@
         </is>
       </c>
       <c r="J67" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="42" customHeight="1">
+      <c r="A68" s="16" t="inlineStr">
+        <is>
+          <t>#67</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-23 15:33:21 +0530</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>Phase 7: Community Overhaul</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>62aa3ff</t>
+        </is>
+      </c>
+      <c r="F68" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>Prepare a separate file .txt in this project recording changes with timestamps from starting to end.</t>
+        </is>
+      </c>
+      <c r="H68" s="18" t="inlineStr">
+        <is>
+          <t>Created comprehensive chronological CHANGES_LOG.txt and changes.txt documenting all 66 development milestones and 92 commits.</t>
+        </is>
+      </c>
+      <c r="I68" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, changes.txt</t>
+        </is>
+      </c>
+      <c r="J68" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="42" customHeight="1">
+      <c r="A69" s="22" t="inlineStr">
+        <is>
+          <t>#68</t>
+        </is>
+      </c>
+      <c r="B69" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-23 15:37:56 +0530</t>
+        </is>
+      </c>
+      <c r="C69" s="24" t="inlineStr">
+        <is>
+          <t>Phase 7: Community Overhaul</t>
+        </is>
+      </c>
+      <c r="D69" s="22" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E69" s="23" t="inlineStr">
+        <is>
+          <t>8dfe168</t>
+        </is>
+      </c>
+      <c r="F69" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G69" s="24" t="inlineStr">
+        <is>
+          <t>Provide a professional Excel workbook for management and Team Lead (TL) review.</t>
+        </is>
+      </c>
+      <c r="H69" s="24" t="inlineStr">
+        <is>
+          <t>Generated executive 4-sheet formatted Excel workbook (FORGE_Website_Project_Change_Report.xlsx) with KPIs, roadmaps, detailed logs, routes, assets, and companion CSV.</t>
+        </is>
+      </c>
+      <c r="I69" s="26" t="inlineStr">
+        <is>
+          <t>FORGE_Website_Project_Change_Report.xlsx, FORGE_Website_Project_Change_Report.csv</t>
+        </is>
+      </c>
+      <c r="J69" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="42" customHeight="1">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>#69</t>
+        </is>
+      </c>
+      <c r="B70" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-23 15:50:33 +0530</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>Phase 7: Community Overhaul</t>
+        </is>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E70" s="17" t="inlineStr">
+        <is>
+          <t>LIVE_PROD</t>
+        </is>
+      </c>
+      <c r="F70" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G70" s="18" t="inlineStr">
+        <is>
+          <t>Upload these changes to GitHub and Vercel.</t>
+        </is>
+      </c>
+      <c r="H70" s="18" t="inlineStr">
+        <is>
+          <t>Pushed all latest commits (ea72018, 62aa3ff, 8dfe168) to GitHub main branch; triggered and verified Vercel production deployment at https://winnoforge-website-d1.vercel.app with HTTP/2 200 responses across all routes.</t>
+        </is>
+      </c>
+      <c r="I70" s="20" t="inlineStr">
+        <is>
+          <t>GitHub origin/main, Vercel Production Deployment</t>
+        </is>
+      </c>
+      <c r="J70" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat(automation): add auto_update_changelogs.py and configure recurring 2-hour cron synchronization for Excel and txt records
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -107,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -143,11 +143,55 @@
         <color rgb="000B1528"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -223,6 +267,8 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -632,8 +678,8 @@
           <t>YashSri/winnoforge_website_d1</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="28" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -646,8 +692,8 @@
           <t>main (Clean / Production Ready)</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="28" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -657,11 +703,11 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>92 Commits Recorded</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
+          <t>95 Commits Recorded</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="28" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -671,11 +717,11 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>66 Actionable Milestones</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
+          <t>95 Actionable Milestones</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="28" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -688,8 +734,8 @@
           <t>8 Primary + Dynamic [slug]</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
+      <c r="C9" s="27" t="n"/>
+      <c r="D9" s="28" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -702,8 +748,8 @@
           <t>0 Errors (npx tsc --noEmit)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
+      <c r="C10" s="27" t="n"/>
+      <c r="D10" s="28" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -716,8 +762,8 @@
           <t>19/19 Routes Passed (npm run build)</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
+      <c r="C11" s="27" t="n"/>
+      <c r="D11" s="28" t="n"/>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -991,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4641,6 +4687,1410 @@
         </is>
       </c>
       <c r="J70" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="22" t="inlineStr">
+        <is>
+          <t>#70</t>
+        </is>
+      </c>
+      <c r="B71" s="23" t="inlineStr">
+        <is>
+          <t>2026-04-21 15:06:46 +0530</t>
+        </is>
+      </c>
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D71" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E71" s="23" t="inlineStr">
+        <is>
+          <t>baf28d4</t>
+        </is>
+      </c>
+      <c r="F71" s="25" t="inlineStr">
+        <is>
+          <t>tanishqsharma24</t>
+        </is>
+      </c>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="H71" s="24" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="I71" s="26" t="inlineStr">
+        <is>
+          <t>app/citadel1/page.tsx, app/community/page.tsx, app/impact/page.tsx, app/institution/page.tsx, app/page.tsx (+45 more)</t>
+        </is>
+      </c>
+      <c r="J71" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="40" customHeight="1">
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>#71</t>
+        </is>
+      </c>
+      <c r="B72" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:19:47 +0530</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E72" s="17" t="inlineStr">
+        <is>
+          <t>8692ecf</t>
+        </is>
+      </c>
+      <c r="F72" s="19" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="inlineStr">
+        <is>
+          <t>Remove dead cert/Supabase residue from winnoforge-main1</t>
+        </is>
+      </c>
+      <c r="H72" s="18" t="inlineStr">
+        <is>
+          <t>Remove dead cert/Supabase residue from winnoforge-main1</t>
+        </is>
+      </c>
+      <c r="I72" s="20" t="inlineStr">
+        <is>
+          <t>.../winnoforge-main1/app/api/cert/admin/route.ts, .../app/api/cert/certificates/[id]/qrcode/route.ts, .../app/api/cert/certificates/[id]/revoke/route.ts, .../app/api/cert/certificates/route.ts, .../winnoforge-main1/app/api/cert/upload/route.ts (+8 more)</t>
+        </is>
+      </c>
+      <c r="J72" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="40" customHeight="1">
+      <c r="A73" s="22" t="inlineStr">
+        <is>
+          <t>#72</t>
+        </is>
+      </c>
+      <c r="B73" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:29:32 +0530</t>
+        </is>
+      </c>
+      <c r="C73" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D73" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E73" s="23" t="inlineStr">
+        <is>
+          <t>cc6a450</t>
+        </is>
+      </c>
+      <c r="F73" s="25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G73" s="24" t="inlineStr">
+        <is>
+          <t>Wire gated-download modal into program catalog and detail pages</t>
+        </is>
+      </c>
+      <c r="H73" s="24" t="inlineStr">
+        <is>
+          <t>Wire gated-download modal into program catalog and detail pages</t>
+        </is>
+      </c>
+      <c r="I73" s="26" t="inlineStr">
+        <is>
+          <t>components/programs/ProgramCard.tsx</t>
+        </is>
+      </c>
+      <c r="J73" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="40" customHeight="1">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>#73</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:34:51 +0530</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E74" s="17" t="inlineStr">
+        <is>
+          <t>6a5f02e</t>
+        </is>
+      </c>
+      <c r="F74" s="19" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>Fix VoicesCarousel layout for non-3-multiple item counts</t>
+        </is>
+      </c>
+      <c r="H74" s="18" t="inlineStr">
+        <is>
+          <t>Fix VoicesCarousel layout for non-3-multiple item counts</t>
+        </is>
+      </c>
+      <c r="I74" s="20" t="inlineStr">
+        <is>
+          <t>components/shared/VoicesCarousel.tsx</t>
+        </is>
+      </c>
+      <c r="J74" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="40" customHeight="1">
+      <c r="A75" s="22" t="inlineStr">
+        <is>
+          <t>#74</t>
+        </is>
+      </c>
+      <c r="B75" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:39:17 +0530</t>
+        </is>
+      </c>
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E75" s="23" t="inlineStr">
+        <is>
+          <t>9e84301</t>
+        </is>
+      </c>
+      <c r="F75" s="25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G75" s="24" t="inlineStr">
+        <is>
+          <t>Add mentor modal type for Become a Mentor CTA</t>
+        </is>
+      </c>
+      <c r="H75" s="24" t="inlineStr">
+        <is>
+          <t>Add mentor modal type for Become a Mentor CTA</t>
+        </is>
+      </c>
+      <c r="I75" s="26" t="inlineStr">
+        <is>
+          <t>app/api/contact/route.ts, components/modal/FormModal.tsx, components/modal/MentorForm.tsx, components/modal/ModalContext.tsx</t>
+        </is>
+      </c>
+      <c r="J75" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>#75</t>
+        </is>
+      </c>
+      <c r="B76" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:05:49 +0530</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E76" s="17" t="inlineStr">
+        <is>
+          <t>cea27fb</t>
+        </is>
+      </c>
+      <c r="F76" s="19" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G76" s="18" t="inlineStr">
+        <is>
+          <t>Fold mentor directory into Community page</t>
+        </is>
+      </c>
+      <c r="H76" s="18" t="inlineStr">
+        <is>
+          <t>Fold mentor directory into Community page</t>
+        </is>
+      </c>
+      <c r="I76" s="20" t="inlineStr">
+        <is>
+          <t>app/mentors/page.tsx, components/community/MentorsSection.tsx, .../components1/community/page (1).tsx</t>
+        </is>
+      </c>
+      <c r="J76" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="22" t="inlineStr">
+        <is>
+          <t>#76</t>
+        </is>
+      </c>
+      <c r="B77" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:09:00 +0530</t>
+        </is>
+      </c>
+      <c r="C77" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E77" s="23" t="inlineStr">
+        <is>
+          <t>b2c83da</t>
+        </is>
+      </c>
+      <c r="F77" s="25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G77" s="24" t="inlineStr">
+        <is>
+          <t>Point stale /corporate links at /collaborate directly</t>
+        </is>
+      </c>
+      <c r="H77" s="24" t="inlineStr">
+        <is>
+          <t>Point stale /corporate links at /collaborate directly</t>
+        </is>
+      </c>
+      <c r="I77" s="26" t="inlineStr">
+        <is>
+          <t>components/Philosophy.tsx, components/home/OfferingsGrid.tsx</t>
+        </is>
+      </c>
+      <c r="J77" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="16" t="inlineStr">
+        <is>
+          <t>#77</t>
+        </is>
+      </c>
+      <c r="B78" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:10:45 +0530</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E78" s="17" t="inlineStr">
+        <is>
+          <t>1e1a501</t>
+        </is>
+      </c>
+      <c r="F78" s="19" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G78" s="18" t="inlineStr">
+        <is>
+          <t>Add Learning Journey timeline to homepage</t>
+        </is>
+      </c>
+      <c r="H78" s="18" t="inlineStr">
+        <is>
+          <t>Add Learning Journey timeline to homepage</t>
+        </is>
+      </c>
+      <c r="I78" s="20" t="inlineStr">
+        <is>
+          <t>app/page.tsx</t>
+        </is>
+      </c>
+      <c r="J78" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="A79" s="22" t="inlineStr">
+        <is>
+          <t>#78</t>
+        </is>
+      </c>
+      <c r="B79" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:14:56 +0530</t>
+        </is>
+      </c>
+      <c r="C79" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E79" s="23" t="inlineStr">
+        <is>
+          <t>1c281b3</t>
+        </is>
+      </c>
+      <c r="F79" s="25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G79" s="24" t="inlineStr">
+        <is>
+          <t>Add Experts &amp; Speakers and Built Through FORGE sections</t>
+        </is>
+      </c>
+      <c r="H79" s="24" t="inlineStr">
+        <is>
+          <t>Add Experts &amp; Speakers and Built Through FORGE sections</t>
+        </is>
+      </c>
+      <c r="I79" s="26" t="inlineStr">
+        <is>
+          <t>app/page.tsx, components/home/BuiltThroughForge.tsx, components/home/ExpertsSpeakers.tsx, lib/experts-data.ts, lib/projects-data.ts</t>
+        </is>
+      </c>
+      <c r="J79" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>#79</t>
+        </is>
+      </c>
+      <c r="B80" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:16:08 +0530</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E80" s="17" t="inlineStr">
+        <is>
+          <t>dd0154b</t>
+        </is>
+      </c>
+      <c r="F80" s="19" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G80" s="18" t="inlineStr">
+        <is>
+          <t>Add Citadel Preview and Community Highlights sections; reposition Voices</t>
+        </is>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>Add Citadel Preview and Community Highlights sections; reposition Voices</t>
+        </is>
+      </c>
+      <c r="I80" s="20" t="inlineStr">
+        <is>
+          <t>app/page.tsx, components/home/CitadelPreview.tsx, components/home/CommunityHighlights.tsx</t>
+        </is>
+      </c>
+      <c r="J80" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="22" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="B81" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:17:40 +0530</t>
+        </is>
+      </c>
+      <c r="C81" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E81" s="23" t="inlineStr">
+        <is>
+          <t>b793717</t>
+        </is>
+      </c>
+      <c r="F81" s="25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G81" s="24" t="inlineStr">
+        <is>
+          <t>Add Final CTA section and homepage SEO metadata</t>
+        </is>
+      </c>
+      <c r="H81" s="24" t="inlineStr">
+        <is>
+          <t>Add Final CTA section and homepage SEO metadata</t>
+        </is>
+      </c>
+      <c r="I81" s="26" t="inlineStr">
+        <is>
+          <t>app/layout.tsx, app/page.tsx, components/home/FinalCta.tsx</t>
+        </is>
+      </c>
+      <c r="J81" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>#81</t>
+        </is>
+      </c>
+      <c r="B82" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:27:55 +0530</t>
+        </is>
+      </c>
+      <c r="C82" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D82" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E82" s="17" t="inlineStr">
+        <is>
+          <t>282b7cc</t>
+        </is>
+      </c>
+      <c r="F82" s="19" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G82" s="18" t="inlineStr">
+        <is>
+          <t>Add SEO metadata to the About &amp; Ecosystem page</t>
+        </is>
+      </c>
+      <c r="H82" s="18" t="inlineStr">
+        <is>
+          <t>Add SEO metadata to the About &amp; Ecosystem page</t>
+        </is>
+      </c>
+      <c r="I82" s="20" t="inlineStr">
+        <is>
+          <t>app/ecosystem/page.tsx, components/winnoforge-main1/app/ecosystem/page.tsx</t>
+        </is>
+      </c>
+      <c r="J82" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="22" t="inlineStr">
+        <is>
+          <t>#82</t>
+        </is>
+      </c>
+      <c r="B83" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:50:20 +0530</t>
+        </is>
+      </c>
+      <c r="C83" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E83" s="23" t="inlineStr">
+        <is>
+          <t>7f2fbe3</t>
+        </is>
+      </c>
+      <c r="F83" s="25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G83" s="24" t="inlineStr">
+        <is>
+          <t>Implement full Mentors &amp; Experts page as its own standalone page</t>
+        </is>
+      </c>
+      <c r="H83" s="24" t="inlineStr">
+        <is>
+          <t>Implement full Mentors &amp; Experts page as its own standalone page</t>
+        </is>
+      </c>
+      <c r="I83" s="26" t="inlineStr">
+        <is>
+          <t>app/api/contact/route.ts, app/mentors/page.tsx, components/citadel/CitadelFinalCta.tsx, components/citadel/MentorshipInside.tsx, components/community/MentorsSection.tsx (+15 more)</t>
+        </is>
+      </c>
+      <c r="J83" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="16" t="inlineStr">
+        <is>
+          <t>#83</t>
+        </is>
+      </c>
+      <c r="B84" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 06:51:16 +0000</t>
+        </is>
+      </c>
+      <c r="C84" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D84" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E84" s="17" t="inlineStr">
+        <is>
+          <t>dc6176d</t>
+        </is>
+      </c>
+      <c r="F84" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G84" s="18" t="inlineStr">
+        <is>
+          <t>Move Stats section to appear right after Hero</t>
+        </is>
+      </c>
+      <c r="H84" s="18" t="inlineStr">
+        <is>
+          <t>Move Stats section to appear right after Hero</t>
+        </is>
+      </c>
+      <c r="I84" s="20" t="inlineStr">
+        <is>
+          <t>app/page.tsx</t>
+        </is>
+      </c>
+      <c r="J84" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="22" t="inlineStr">
+        <is>
+          <t>#84</t>
+        </is>
+      </c>
+      <c r="B85" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:49:24 +0000</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D85" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E85" s="23" t="inlineStr">
+        <is>
+          <t>c68b56d</t>
+        </is>
+      </c>
+      <c r="F85" s="25" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G85" s="24" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/main' into claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="H85" s="24" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/main' into claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="I85" s="26" t="inlineStr">
+        <is>
+          <t>, app/api/contact/route.ts, app/collaborate/layout.tsx, app/collaborate/page.tsx, app/corporate/page.tsx (+122 more)</t>
+        </is>
+      </c>
+      <c r="J85" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="16" t="inlineStr">
+        <is>
+          <t>#85</t>
+        </is>
+      </c>
+      <c r="B86" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:51:28 +0000</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E86" s="17" t="inlineStr">
+        <is>
+          <t>6a5c0bb</t>
+        </is>
+      </c>
+      <c r="F86" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G86" s="18" t="inlineStr">
+        <is>
+          <t>Fix lint: sort imports and format Stats/page after merge</t>
+        </is>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>Fix lint: sort imports and format Stats/page after merge</t>
+        </is>
+      </c>
+      <c r="I86" s="20" t="inlineStr">
+        <is>
+          <t>app/page.tsx, components/Stats.tsx</t>
+        </is>
+      </c>
+      <c r="J86" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>#86</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 21:22:04 +0530</t>
+        </is>
+      </c>
+      <c r="C87" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D87" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E87" s="23" t="inlineStr">
+        <is>
+          <t>a8f989c</t>
+        </is>
+      </c>
+      <c r="F87" s="25" t="inlineStr">
+        <is>
+          <t>tanishqsharma24</t>
+        </is>
+      </c>
+      <c r="G87" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #1 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="H87" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #1 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="I87" s="26" t="inlineStr">
+        <is>
+          <t>, app/page.tsx, components/Stats.tsx</t>
+        </is>
+      </c>
+      <c r="J87" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="16" t="inlineStr">
+        <is>
+          <t>#87</t>
+        </is>
+      </c>
+      <c r="B88" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 23:15:42 +0530</t>
+        </is>
+      </c>
+      <c r="C88" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D88" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E88" s="17" t="inlineStr">
+        <is>
+          <t>651568b</t>
+        </is>
+      </c>
+      <c r="F88" s="19" t="inlineStr">
+        <is>
+          <t>tanishqsharma24</t>
+        </is>
+      </c>
+      <c r="G88" s="18" t="inlineStr">
+        <is>
+          <t>Merge pull request #2 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="H88" s="18" t="inlineStr">
+        <is>
+          <t>Merge pull request #2 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="I88" s="20" t="inlineStr">
+        <is>
+          <t>, components/Stats.tsx</t>
+        </is>
+      </c>
+      <c r="J88" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="22" t="inlineStr">
+        <is>
+          <t>#88</t>
+        </is>
+      </c>
+      <c r="B89" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 17:51:19 +0000</t>
+        </is>
+      </c>
+      <c r="C89" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D89" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E89" s="23" t="inlineStr">
+        <is>
+          <t>9ac260e</t>
+        </is>
+      </c>
+      <c r="F89" s="25" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G89" s="24" t="inlineStr">
+        <is>
+          <t>Use brand palette colors for the FORGE Citadel offering card</t>
+        </is>
+      </c>
+      <c r="H89" s="24" t="inlineStr">
+        <is>
+          <t>Use brand palette colors for the FORGE Citadel offering card</t>
+        </is>
+      </c>
+      <c r="I89" s="26" t="inlineStr">
+        <is>
+          <t>components/home/OfferingsGrid.tsx</t>
+        </is>
+      </c>
+      <c r="J89" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="16" t="inlineStr">
+        <is>
+          <t>#89</t>
+        </is>
+      </c>
+      <c r="B90" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-16 17:51:41 +0000</t>
+        </is>
+      </c>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E90" s="17" t="inlineStr">
+        <is>
+          <t>bd80955</t>
+        </is>
+      </c>
+      <c r="F90" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G90" s="18" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/main' into claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>Merge remote-tracking branch 'origin/main' into claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="I90" s="20" t="inlineStr">
+        <is>
+          <t>Repository root</t>
+        </is>
+      </c>
+      <c r="J90" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="22" t="inlineStr">
+        <is>
+          <t>#90</t>
+        </is>
+      </c>
+      <c r="B91" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-16 23:22:13 +0530</t>
+        </is>
+      </c>
+      <c r="C91" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E91" s="23" t="inlineStr">
+        <is>
+          <t>19bb787</t>
+        </is>
+      </c>
+      <c r="F91" s="25" t="inlineStr">
+        <is>
+          <t>tanishqsharma24</t>
+        </is>
+      </c>
+      <c r="G91" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #3 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="H91" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #3 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="I91" s="26" t="inlineStr">
+        <is>
+          <t>, components/home/OfferingsGrid.tsx</t>
+        </is>
+      </c>
+      <c r="J91" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="16" t="inlineStr">
+        <is>
+          <t>#91</t>
+        </is>
+      </c>
+      <c r="B92" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-17 03:23:29 +0000</t>
+        </is>
+      </c>
+      <c r="C92" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D92" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E92" s="17" t="inlineStr">
+        <is>
+          <t>e8e72e7</t>
+        </is>
+      </c>
+      <c r="F92" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G92" s="18" t="inlineStr">
+        <is>
+          <t>Make Philosophy section's scroll animation smoother and faster</t>
+        </is>
+      </c>
+      <c r="H92" s="18" t="inlineStr">
+        <is>
+          <t>Make Philosophy section's scroll animation smoother and faster</t>
+        </is>
+      </c>
+      <c r="I92" s="20" t="inlineStr">
+        <is>
+          <t>components/Philosophy.tsx</t>
+        </is>
+      </c>
+      <c r="J92" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="40" customHeight="1">
+      <c r="A93" s="22" t="inlineStr">
+        <is>
+          <t>#92</t>
+        </is>
+      </c>
+      <c r="B93" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-17 08:53:40 +0530</t>
+        </is>
+      </c>
+      <c r="C93" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D93" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E93" s="23" t="inlineStr">
+        <is>
+          <t>8533458</t>
+        </is>
+      </c>
+      <c r="F93" s="25" t="inlineStr">
+        <is>
+          <t>tanishqsharma24</t>
+        </is>
+      </c>
+      <c r="G93" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #4 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="H93" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #4 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="I93" s="26" t="inlineStr">
+        <is>
+          <t>, components/Philosophy.tsx</t>
+        </is>
+      </c>
+      <c r="J93" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="40" customHeight="1">
+      <c r="A94" s="16" t="inlineStr">
+        <is>
+          <t>#93</t>
+        </is>
+      </c>
+      <c r="B94" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-17 03:26:05 +0000</t>
+        </is>
+      </c>
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D94" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E94" s="17" t="inlineStr">
+        <is>
+          <t>9dbb8e4</t>
+        </is>
+      </c>
+      <c r="F94" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G94" s="18" t="inlineStr">
+        <is>
+          <t>Revert Philosophy scroll animation tuning</t>
+        </is>
+      </c>
+      <c r="H94" s="18" t="inlineStr">
+        <is>
+          <t>Revert Philosophy scroll animation tuning</t>
+        </is>
+      </c>
+      <c r="I94" s="20" t="inlineStr">
+        <is>
+          <t>components/Philosophy.tsx</t>
+        </is>
+      </c>
+      <c r="J94" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="40" customHeight="1">
+      <c r="A95" s="22" t="inlineStr">
+        <is>
+          <t>#94</t>
+        </is>
+      </c>
+      <c r="B95" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-17 08:56:14 +0530</t>
+        </is>
+      </c>
+      <c r="C95" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D95" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E95" s="23" t="inlineStr">
+        <is>
+          <t>fef8fc6</t>
+        </is>
+      </c>
+      <c r="F95" s="25" t="inlineStr">
+        <is>
+          <t>tanishqsharma24</t>
+        </is>
+      </c>
+      <c r="G95" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #5 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="H95" s="24" t="inlineStr">
+        <is>
+          <t>Merge pull request #5 from YashSri/claude/affectionate-turing-knks9g</t>
+        </is>
+      </c>
+      <c r="I95" s="26" t="inlineStr">
+        <is>
+          <t>, components/Philosophy.tsx</t>
+        </is>
+      </c>
+      <c r="J95" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="40" customHeight="1">
+      <c r="A96" s="16" t="inlineStr">
+        <is>
+          <t>#95</t>
+        </is>
+      </c>
+      <c r="B96" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:20:51 +0530</t>
+        </is>
+      </c>
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D96" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E96" s="17" t="inlineStr">
+        <is>
+          <t>ea582ba</t>
+        </is>
+      </c>
+      <c r="F96" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G96" s="18" t="inlineStr">
+        <is>
+          <t>Restore all changes</t>
+        </is>
+      </c>
+      <c r="H96" s="18" t="inlineStr">
+        <is>
+          <t>Restore all changes</t>
+        </is>
+      </c>
+      <c r="I96" s="20" t="inlineStr">
+        <is>
+          <t>Repository root</t>
+        </is>
+      </c>
+      <c r="J96" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="40" customHeight="1">
+      <c r="A97" s="22" t="inlineStr">
+        <is>
+          <t>#96</t>
+        </is>
+      </c>
+      <c r="B97" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-23 16:49:02 +0530</t>
+        </is>
+      </c>
+      <c r="C97" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D97" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E97" s="23" t="inlineStr">
+        <is>
+          <t>505f983</t>
+        </is>
+      </c>
+      <c r="F97" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G97" s="24" t="inlineStr">
+        <is>
+          <t>docs: update CHANGES_LOG.txt and changes.txt with GitHub push and Vercel production deployment records</t>
+        </is>
+      </c>
+      <c r="H97" s="24" t="inlineStr">
+        <is>
+          <t>docs: update CHANGES_LOG.txt and changes.txt with GitHub push and Vercel production deployment records</t>
+        </is>
+      </c>
+      <c r="I97" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J97" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs(changelog): record collaborate hero redesign in logs and excel report
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>96 Commits Recorded</t>
+          <t>98 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>96 Actionable Milestones</t>
+          <t>98 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J98"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6143,6 +6143,110 @@
         </is>
       </c>
       <c r="J98" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="40" customHeight="1">
+      <c r="A99" s="22" t="inlineStr">
+        <is>
+          <t>#98</t>
+        </is>
+      </c>
+      <c r="B99" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:44:18 +0530</t>
+        </is>
+      </c>
+      <c r="C99" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D99" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E99" s="23" t="inlineStr">
+        <is>
+          <t>f7edfe4</t>
+        </is>
+      </c>
+      <c r="F99" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G99" s="24" t="inlineStr">
+        <is>
+          <t>chore(sync): automated changelog synchronization (iteration 1)</t>
+        </is>
+      </c>
+      <c r="H99" s="24" t="inlineStr">
+        <is>
+          <t>chore(sync): automated changelog synchronization (iteration 1)</t>
+        </is>
+      </c>
+      <c r="I99" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J99" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="40" customHeight="1">
+      <c r="A100" s="16" t="inlineStr">
+        <is>
+          <t>#99</t>
+        </is>
+      </c>
+      <c r="B100" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 11:22:18 +0530</t>
+        </is>
+      </c>
+      <c r="C100" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D100" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E100" s="17" t="inlineStr">
+        <is>
+          <t>7747db3</t>
+        </is>
+      </c>
+      <c r="F100" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G100" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign collaborate hero with swiss editorial layout, ambient motion, and line-based reveals</t>
+        </is>
+      </c>
+      <c r="H100" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign collaborate hero with swiss editorial layout, ambient motion, and line-based reveals</t>
+        </is>
+      </c>
+      <c r="I100" s="20" t="inlineStr">
+        <is>
+          <t>app/collaborate/page.tsx, app/globals.css, components/collaborate/CollaborateHero.tsx</t>
+        </is>
+      </c>
+      <c r="J100" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs(changelog): update local logs and excel report for collaboration pathways redesign
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>98 Commits Recorded</t>
+          <t>100 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>98 Actionable Milestones</t>
+          <t>100 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6247,6 +6247,110 @@
         </is>
       </c>
       <c r="J100" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="40" customHeight="1">
+      <c r="A101" s="22" t="inlineStr">
+        <is>
+          <t>#100</t>
+        </is>
+      </c>
+      <c r="B101" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 11:24:24 +0530</t>
+        </is>
+      </c>
+      <c r="C101" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D101" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E101" s="23" t="inlineStr">
+        <is>
+          <t>0675cc2</t>
+        </is>
+      </c>
+      <c r="F101" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G101" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): record collaborate hero redesign in logs and excel report</t>
+        </is>
+      </c>
+      <c r="H101" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): record collaborate hero redesign in logs and excel report</t>
+        </is>
+      </c>
+      <c r="I101" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J101" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="40" customHeight="1">
+      <c r="A102" s="16" t="inlineStr">
+        <is>
+          <t>#101</t>
+        </is>
+      </c>
+      <c r="B102" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 12:07:17 +0530</t>
+        </is>
+      </c>
+      <c r="C102" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D102" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E102" s="17" t="inlineStr">
+        <is>
+          <t>5473ee5</t>
+        </is>
+      </c>
+      <c r="F102" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G102" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign collaboration pathways section with asymmetric editorial grid, real photography and secondary pathway row</t>
+        </is>
+      </c>
+      <c r="H102" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign collaboration pathways section with asymmetric editorial grid, real photography and secondary pathway row</t>
+        </is>
+      </c>
+      <c r="I102" s="20" t="inlineStr">
+        <is>
+          <t>app/collaborate/page.tsx, components/collaborate/CollaborationPathways.tsx, public/collaborate/pathway-community.jpg, public/collaborate/pathway-founder.jpg, public/collaborate/pathway-industry.jpg (+3 more)</t>
+        </is>
+      </c>
+      <c r="J102" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs(changelog): record partner with forge redesign in local changelogs and excel report
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>100 Commits Recorded</t>
+          <t>102 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>100 Actionable Milestones</t>
+          <t>102 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J102"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6351,6 +6351,110 @@
         </is>
       </c>
       <c r="J102" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="40" customHeight="1">
+      <c r="A103" s="22" t="inlineStr">
+        <is>
+          <t>#102</t>
+        </is>
+      </c>
+      <c r="B103" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 12:11:51 +0530</t>
+        </is>
+      </c>
+      <c r="C103" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D103" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E103" s="23" t="inlineStr">
+        <is>
+          <t>b6c6820</t>
+        </is>
+      </c>
+      <c r="F103" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G103" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update local logs and excel report for collaboration pathways redesign</t>
+        </is>
+      </c>
+      <c r="H103" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update local logs and excel report for collaboration pathways redesign</t>
+        </is>
+      </c>
+      <c r="I103" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J103" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="40" customHeight="1">
+      <c r="A104" s="16" t="inlineStr">
+        <is>
+          <t>#103</t>
+        </is>
+      </c>
+      <c r="B104" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 12:30:44 +0530</t>
+        </is>
+      </c>
+      <c r="C104" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E104" s="17" t="inlineStr">
+        <is>
+          <t>8d5b58c</t>
+        </is>
+      </c>
+      <c r="F104" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G104" s="18" t="inlineStr">
+        <is>
+          <t>feat(partner): redesign partner with forge section with segmented toggle, asymmetric card grid, and editorial photography</t>
+        </is>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
+        <is>
+          <t>feat(partner): redesign partner with forge section with segmented toggle, asymmetric card grid, and editorial photography</t>
+        </is>
+      </c>
+      <c r="I104" s="20" t="inlineStr">
+        <is>
+          <t>app/collaborate/page.tsx, components/partner/PartnerAudienceSection.tsx, components/partner/PartnerWithForge.tsx, public/partner/ind-card-01.jpg, public/partner/ind-card-02.jpg (+10 more)</t>
+        </is>
+      </c>
+      <c r="J104" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report with Collaboration Formats redesign
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>102 Commits Recorded</t>
+          <t>104 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>102 Actionable Milestones</t>
+          <t>104 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J104"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6455,6 +6455,110 @@
         </is>
       </c>
       <c r="J104" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="40" customHeight="1">
+      <c r="A105" s="22" t="inlineStr">
+        <is>
+          <t>#104</t>
+        </is>
+      </c>
+      <c r="B105" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 12:34:08 +0530</t>
+        </is>
+      </c>
+      <c r="C105" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D105" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E105" s="23" t="inlineStr">
+        <is>
+          <t>809f7bd</t>
+        </is>
+      </c>
+      <c r="F105" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G105" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): record partner with forge redesign in local changelogs and excel report</t>
+        </is>
+      </c>
+      <c r="H105" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): record partner with forge redesign in local changelogs and excel report</t>
+        </is>
+      </c>
+      <c r="I105" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J105" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="40" customHeight="1">
+      <c r="A106" s="16" t="inlineStr">
+        <is>
+          <t>#105</t>
+        </is>
+      </c>
+      <c r="B106" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:05:36 +0530</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D106" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E106" s="17" t="inlineStr">
+        <is>
+          <t>42e0c05</t>
+        </is>
+      </c>
+      <c r="F106" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G106" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign Possible Collaboration Formats section with Apple-inspired Uiverse slide-up panels</t>
+        </is>
+      </c>
+      <c r="H106" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign Possible Collaboration Formats section with Apple-inspired Uiverse slide-up panels</t>
+        </is>
+      </c>
+      <c r="I106" s="20" t="inlineStr">
+        <is>
+          <t>app/collaborate/page.tsx, components/collaborate/CollaborationFormats.tsx, public/formats/format-01.jpg, public/formats/format-02.jpg, public/formats/format-03.jpg (+6 more)</t>
+        </is>
+      </c>
+      <c r="J106" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report with Readiness Checklist redesign
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>104 Commits Recorded</t>
+          <t>106 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>104 Actionable Milestones</t>
+          <t>106 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6559,6 +6559,110 @@
         </is>
       </c>
       <c r="J106" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="40" customHeight="1">
+      <c r="A107" s="22" t="inlineStr">
+        <is>
+          <t>#106</t>
+        </is>
+      </c>
+      <c r="B107" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:06:13 +0530</t>
+        </is>
+      </c>
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D107" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E107" s="23" t="inlineStr">
+        <is>
+          <t>839aadc</t>
+        </is>
+      </c>
+      <c r="F107" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G107" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with Collaboration Formats redesign</t>
+        </is>
+      </c>
+      <c r="H107" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with Collaboration Formats redesign</t>
+        </is>
+      </c>
+      <c r="I107" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J107" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="40" customHeight="1">
+      <c r="A108" s="16" t="inlineStr">
+        <is>
+          <t>#107</t>
+        </is>
+      </c>
+      <c r="B108" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:26:54 +0530</t>
+        </is>
+      </c>
+      <c r="C108" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D108" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E108" s="17" t="inlineStr">
+        <is>
+          <t>b73ac8f</t>
+        </is>
+      </c>
+      <c r="F108" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G108" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign Collaboration Readiness Checklist with 4x2 editorial grid and alternating slide-in panels</t>
+        </is>
+      </c>
+      <c r="H108" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign Collaboration Readiness Checklist with 4x2 editorial grid and alternating slide-in panels</t>
+        </is>
+      </c>
+      <c r="I108" s="20" t="inlineStr">
+        <is>
+          <t>components/collaborate/ReadinessChecklist.tsx, public/checklist/checklist-01.jpg, public/checklist/checklist-02.jpg, public/checklist/checklist-03.jpg, public/checklist/checklist-04.jpg (+4 more)</t>
+        </is>
+      </c>
+      <c r="J108" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report after removing bottom collaborate CTA section
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>106 Commits Recorded</t>
+          <t>108 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>106 Actionable Milestones</t>
+          <t>108 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6663,6 +6663,110 @@
         </is>
       </c>
       <c r="J108" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="40" customHeight="1">
+      <c r="A109" s="22" t="inlineStr">
+        <is>
+          <t>#108</t>
+        </is>
+      </c>
+      <c r="B109" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:27:30 +0530</t>
+        </is>
+      </c>
+      <c r="C109" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D109" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E109" s="23" t="inlineStr">
+        <is>
+          <t>02c9638</t>
+        </is>
+      </c>
+      <c r="F109" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G109" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with Readiness Checklist redesign</t>
+        </is>
+      </c>
+      <c r="H109" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with Readiness Checklist redesign</t>
+        </is>
+      </c>
+      <c r="I109" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J109" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="40" customHeight="1">
+      <c r="A110" s="16" t="inlineStr">
+        <is>
+          <t>#109</t>
+        </is>
+      </c>
+      <c r="B110" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:39:44 +0530</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D110" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E110" s="17" t="inlineStr">
+        <is>
+          <t>04b2ec1</t>
+        </is>
+      </c>
+      <c r="F110" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G110" s="18" t="inlineStr">
+        <is>
+          <t>refactor(collaborate): remove redundant Have an Idea for Collaboration section</t>
+        </is>
+      </c>
+      <c r="H110" s="18" t="inlineStr">
+        <is>
+          <t>refactor(collaborate): remove redundant Have an Idea for Collaboration section</t>
+        </is>
+      </c>
+      <c r="I110" s="20" t="inlineStr">
+        <is>
+          <t>app/collaborate/page.tsx</t>
+        </is>
+      </c>
+      <c r="J110" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report with Get In Touch section redesign
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>108 Commits Recorded</t>
+          <t>110 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>108 Actionable Milestones</t>
+          <t>110 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6767,6 +6767,110 @@
         </is>
       </c>
       <c r="J110" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="40" customHeight="1">
+      <c r="A111" s="22" t="inlineStr">
+        <is>
+          <t>#110</t>
+        </is>
+      </c>
+      <c r="B111" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:40:41 +0530</t>
+        </is>
+      </c>
+      <c r="C111" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D111" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E111" s="23" t="inlineStr">
+        <is>
+          <t>fddcdc4</t>
+        </is>
+      </c>
+      <c r="F111" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G111" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report after removing bottom collaborate CTA section</t>
+        </is>
+      </c>
+      <c r="H111" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report after removing bottom collaborate CTA section</t>
+        </is>
+      </c>
+      <c r="I111" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J111" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="40" customHeight="1">
+      <c r="A112" s="16" t="inlineStr">
+        <is>
+          <t>#111</t>
+        </is>
+      </c>
+      <c r="B112" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:57:43 +0530</t>
+        </is>
+      </c>
+      <c r="C112" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D112" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E112" s="17" t="inlineStr">
+        <is>
+          <t>28a9857</t>
+        </is>
+      </c>
+      <c r="F112" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G112" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign Get In Touch section with two-column editorial layout and subtle glass enquiry form</t>
+        </is>
+      </c>
+      <c r="H112" s="18" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign Get In Touch section with two-column editorial layout and subtle glass enquiry form</t>
+        </is>
+      </c>
+      <c r="I112" s="20" t="inlineStr">
+        <is>
+          <t>app/collaborate/page.tsx, components/collaborate/CollaborateForm.tsx, public/collaborate/get-in-touch-campus.jpg</t>
+        </is>
+      </c>
+      <c r="J112" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report after navbar glass upgrade
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>111 Commits Recorded</t>
+          <t>113 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>111 Actionable Milestones</t>
+          <t>113 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6923,6 +6923,110 @@
         </is>
       </c>
       <c r="J113" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="40" customHeight="1">
+      <c r="A114" s="16" t="inlineStr">
+        <is>
+          <t>#113</t>
+        </is>
+      </c>
+      <c r="B114" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:00:50 +0530</t>
+        </is>
+      </c>
+      <c r="C114" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D114" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E114" s="17" t="inlineStr">
+        <is>
+          <t>c2bd11e</t>
+        </is>
+      </c>
+      <c r="F114" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G114" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync automated changelog and executive Excel report</t>
+        </is>
+      </c>
+      <c r="H114" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync automated changelog and executive Excel report</t>
+        </is>
+      </c>
+      <c r="I114" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J114" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="40" customHeight="1">
+      <c r="A115" s="22" t="inlineStr">
+        <is>
+          <t>#114</t>
+        </is>
+      </c>
+      <c r="B115" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:18:09 +0530</t>
+        </is>
+      </c>
+      <c r="C115" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D115" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E115" s="23" t="inlineStr">
+        <is>
+          <t>daa4392</t>
+        </is>
+      </c>
+      <c r="F115" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G115" s="24" t="inlineStr">
+        <is>
+          <t>feat(navbar): implement premium glass navigation with sliding active pill and inner highlights</t>
+        </is>
+      </c>
+      <c r="H115" s="24" t="inlineStr">
+        <is>
+          <t>feat(navbar): implement premium glass navigation with sliding active pill and inner highlights</t>
+        </is>
+      </c>
+      <c r="I115" s="26" t="inlineStr">
+        <is>
+          <t>components/Navbar.tsx</t>
+        </is>
+      </c>
+      <c r="J115" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report with liquid glass navbar and form updates
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>113 Commits Recorded</t>
+          <t>115 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>113 Actionable Milestones</t>
+          <t>115 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7027,6 +7027,110 @@
         </is>
       </c>
       <c r="J115" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="40" customHeight="1">
+      <c r="A116" s="16" t="inlineStr">
+        <is>
+          <t>#115</t>
+        </is>
+      </c>
+      <c r="B116" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:19:03 +0530</t>
+        </is>
+      </c>
+      <c r="C116" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D116" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E116" s="17" t="inlineStr">
+        <is>
+          <t>19e5470</t>
+        </is>
+      </c>
+      <c r="F116" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G116" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report after navbar glass upgrade</t>
+        </is>
+      </c>
+      <c r="H116" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report after navbar glass upgrade</t>
+        </is>
+      </c>
+      <c r="I116" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J116" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="40" customHeight="1">
+      <c r="A117" s="22" t="inlineStr">
+        <is>
+          <t>#116</t>
+        </is>
+      </c>
+      <c r="B117" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:32:02 +0530</t>
+        </is>
+      </c>
+      <c r="C117" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D117" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E117" s="23" t="inlineStr">
+        <is>
+          <t>b62fd0b</t>
+        </is>
+      </c>
+      <c r="F117" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G117" s="24" t="inlineStr">
+        <is>
+          <t>feat(navbar,form): integrate CodeFronts liquid glass floating capsule and scroll collapse physics</t>
+        </is>
+      </c>
+      <c r="H117" s="24" t="inlineStr">
+        <is>
+          <t>feat(navbar,form): integrate CodeFronts liquid glass floating capsule and scroll collapse physics</t>
+        </is>
+      </c>
+      <c r="I117" s="26" t="inlineStr">
+        <is>
+          <t>components/Navbar.tsx, components/collaborate/CollaborateForm.tsx</t>
+        </is>
+      </c>
+      <c r="J117" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report with FORGE liquid glass system
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>115 Commits Recorded</t>
+          <t>117 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>115 Actionable Milestones</t>
+          <t>117 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7131,6 +7131,110 @@
         </is>
       </c>
       <c r="J117" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="40" customHeight="1">
+      <c r="A118" s="16" t="inlineStr">
+        <is>
+          <t>#117</t>
+        </is>
+      </c>
+      <c r="B118" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:34:03 +0530</t>
+        </is>
+      </c>
+      <c r="C118" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D118" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E118" s="17" t="inlineStr">
+        <is>
+          <t>cd508fe</t>
+        </is>
+      </c>
+      <c r="F118" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G118" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with liquid glass navbar and form updates</t>
+        </is>
+      </c>
+      <c r="H118" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with liquid glass navbar and form updates</t>
+        </is>
+      </c>
+      <c r="I118" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J118" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="40" customHeight="1">
+      <c r="A119" s="22" t="inlineStr">
+        <is>
+          <t>#118</t>
+        </is>
+      </c>
+      <c r="B119" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:49:13 +0530</t>
+        </is>
+      </c>
+      <c r="C119" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D119" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E119" s="23" t="inlineStr">
+        <is>
+          <t>5719363</t>
+        </is>
+      </c>
+      <c r="F119" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G119" s="24" t="inlineStr">
+        <is>
+          <t>feat(navbar,form): implement FORGE liquid glass system for navbar and community form</t>
+        </is>
+      </c>
+      <c r="H119" s="24" t="inlineStr">
+        <is>
+          <t>feat(navbar,form): implement FORGE liquid glass system for navbar and community form</t>
+        </is>
+      </c>
+      <c r="I119" s="26" t="inlineStr">
+        <is>
+          <t>app/globals.css, components/Navbar.tsx, components/collaborate/CollaborateForm.tsx</t>
+        </is>
+      </c>
+      <c r="J119" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelogs and Excel report with navbar active pill fix
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>117 Commits Recorded</t>
+          <t>119 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>117 Actionable Milestones</t>
+          <t>119 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7235,6 +7235,110 @@
         </is>
       </c>
       <c r="J119" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="40" customHeight="1">
+      <c r="A120" s="16" t="inlineStr">
+        <is>
+          <t>#119</t>
+        </is>
+      </c>
+      <c r="B120" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:49:55 +0530</t>
+        </is>
+      </c>
+      <c r="C120" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D120" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E120" s="17" t="inlineStr">
+        <is>
+          <t>77da489</t>
+        </is>
+      </c>
+      <c r="F120" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G120" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with FORGE liquid glass system</t>
+        </is>
+      </c>
+      <c r="H120" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with FORGE liquid glass system</t>
+        </is>
+      </c>
+      <c r="I120" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J120" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="40" customHeight="1">
+      <c r="A121" s="22" t="inlineStr">
+        <is>
+          <t>#120</t>
+        </is>
+      </c>
+      <c r="B121" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:57:42 +0530</t>
+        </is>
+      </c>
+      <c r="C121" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D121" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E121" s="23" t="inlineStr">
+        <is>
+          <t>b2d59d0</t>
+        </is>
+      </c>
+      <c r="F121" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G121" s="24" t="inlineStr">
+        <is>
+          <t>fix(navbar): lock active pill alignment on scroll with stable link geometry and ResizeObserver</t>
+        </is>
+      </c>
+      <c r="H121" s="24" t="inlineStr">
+        <is>
+          <t>fix(navbar): lock active pill alignment on scroll with stable link geometry and ResizeObserver</t>
+        </is>
+      </c>
+      <c r="I121" s="26" t="inlineStr">
+        <is>
+          <t>components/Navbar.tsx</t>
+        </is>
+      </c>
+      <c r="J121" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: update changelog and excel change report
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>119 Commits Recorded</t>
+          <t>121 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>119 Actionable Milestones</t>
+          <t>121 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7339,6 +7339,110 @@
         </is>
       </c>
       <c r="J121" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="40" customHeight="1">
+      <c r="A122" s="16" t="inlineStr">
+        <is>
+          <t>#121</t>
+        </is>
+      </c>
+      <c r="B122" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:58:04 +0530</t>
+        </is>
+      </c>
+      <c r="C122" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D122" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E122" s="17" t="inlineStr">
+        <is>
+          <t>2c8b82b</t>
+        </is>
+      </c>
+      <c r="F122" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G122" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with navbar active pill fix</t>
+        </is>
+      </c>
+      <c r="H122" s="18" t="inlineStr">
+        <is>
+          <t>docs: sync changelogs and Excel report with navbar active pill fix</t>
+        </is>
+      </c>
+      <c r="I122" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J122" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="40" customHeight="1">
+      <c r="A123" s="22" t="inlineStr">
+        <is>
+          <t>#122</t>
+        </is>
+      </c>
+      <c r="B123" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:19:02 +0530</t>
+        </is>
+      </c>
+      <c r="C123" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D123" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E123" s="23" t="inlineStr">
+        <is>
+          <t>f226702</t>
+        </is>
+      </c>
+      <c r="F123" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G123" s="24" t="inlineStr">
+        <is>
+          <t>fix(form): center icons and normalize text alignment in collaborate form</t>
+        </is>
+      </c>
+      <c r="H123" s="24" t="inlineStr">
+        <is>
+          <t>fix(form): center icons and normalize text alignment in collaborate form</t>
+        </is>
+      </c>
+      <c r="I123" s="26" t="inlineStr">
+        <is>
+          <t>components/collaborate/CollaborateForm.tsx</t>
+        </is>
+      </c>
+      <c r="J123" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: update changelog and excel report for partner section redesign
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>121 Commits Recorded</t>
+          <t>123 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>121 Actionable Milestones</t>
+          <t>123 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J123"/>
+  <dimension ref="A1:J125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7443,6 +7443,110 @@
         </is>
       </c>
       <c r="J123" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="40" customHeight="1">
+      <c r="A124" s="16" t="inlineStr">
+        <is>
+          <t>#123</t>
+        </is>
+      </c>
+      <c r="B124" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:21:16 +0530</t>
+        </is>
+      </c>
+      <c r="C124" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D124" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E124" s="17" t="inlineStr">
+        <is>
+          <t>1de7993</t>
+        </is>
+      </c>
+      <c r="F124" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G124" s="18" t="inlineStr">
+        <is>
+          <t>docs: update changelog and excel change report</t>
+        </is>
+      </c>
+      <c r="H124" s="18" t="inlineStr">
+        <is>
+          <t>docs: update changelog and excel change report</t>
+        </is>
+      </c>
+      <c r="I124" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J124" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="40" customHeight="1">
+      <c r="A125" s="22" t="inlineStr">
+        <is>
+          <t>#124</t>
+        </is>
+      </c>
+      <c r="B125" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:45:12 +0530</t>
+        </is>
+      </c>
+      <c r="C125" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D125" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E125" s="23" t="inlineStr">
+        <is>
+          <t>b117bfe</t>
+        </is>
+      </c>
+      <c r="F125" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G125" s="24" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign partner &amp; contributor representation section with single row and editorial layout</t>
+        </is>
+      </c>
+      <c r="H125" s="24" t="inlineStr">
+        <is>
+          <t>feat(collaborate): redesign partner &amp; contributor representation section with single row and editorial layout</t>
+        </is>
+      </c>
+      <c r="I125" s="26" t="inlineStr">
+        <is>
+          <t>components/collaborate/PartnerRepresentation.tsx, public/logos/airtel-transparent.png, public/logos/dabur-transparent.png, public/logos/infynix-transparent.png, public/logos/lightstorm-transparent.png (+3 more)</t>
+        </is>
+      </c>
+      <c r="J125" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: finalize changelogs and Excel report for deployment
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>123 Commits Recorded</t>
+          <t>124 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>123 Actionable Milestones</t>
+          <t>124 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J125"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7547,6 +7547,58 @@
         </is>
       </c>
       <c r="J125" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="40" customHeight="1">
+      <c r="A126" s="16" t="inlineStr">
+        <is>
+          <t>#125</t>
+        </is>
+      </c>
+      <c r="B126" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:47:03 +0530</t>
+        </is>
+      </c>
+      <c r="C126" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D126" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E126" s="17" t="inlineStr">
+        <is>
+          <t>8ca6958</t>
+        </is>
+      </c>
+      <c r="F126" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G126" s="18" t="inlineStr">
+        <is>
+          <t>docs: update changelog and excel report for partner section redesign</t>
+        </is>
+      </c>
+      <c r="H126" s="18" t="inlineStr">
+        <is>
+          <t>docs: update changelog and excel report for partner section redesign</t>
+        </is>
+      </c>
+      <c r="I126" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J126" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: update changelog and excel report for supporter logos fix
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>126 Commits Recorded</t>
+          <t>128 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>126 Actionable Milestones</t>
+          <t>128 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:J130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7703,6 +7703,110 @@
         </is>
       </c>
       <c r="J128" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="40" customHeight="1">
+      <c r="A129" s="22" t="inlineStr">
+        <is>
+          <t>#128</t>
+        </is>
+      </c>
+      <c r="B129" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-02 19:51:19 +0530</t>
+        </is>
+      </c>
+      <c r="C129" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D129" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E129" s="23" t="inlineStr">
+        <is>
+          <t>628e0b3</t>
+        </is>
+      </c>
+      <c r="F129" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G129" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync automated changelog and Excel report</t>
+        </is>
+      </c>
+      <c r="H129" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync automated changelog and Excel report</t>
+        </is>
+      </c>
+      <c r="I129" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J129" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="40" customHeight="1">
+      <c r="A130" s="16" t="inlineStr">
+        <is>
+          <t>#129</t>
+        </is>
+      </c>
+      <c r="B130" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-02 20:47:48 +0530</t>
+        </is>
+      </c>
+      <c r="C130" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D130" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E130" s="17" t="inlineStr">
+        <is>
+          <t>c035825</t>
+        </is>
+      </c>
+      <c r="F130" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G130" s="18" t="inlineStr">
+        <is>
+          <t>feat(hero): upgrade supporter and founder logos to high-res transparent assets without background boxes</t>
+        </is>
+      </c>
+      <c r="H130" s="18" t="inlineStr">
+        <is>
+          <t>feat(hero): upgrade supporter and founder logos to high-res transparent assets without background boxes</t>
+        </is>
+      </c>
+      <c r="I130" s="20" t="inlineStr">
+        <is>
+          <t>components/Hero.tsx, public/supporters/faceoff-clean.png, public/supporters/faceoff.png, public/supporters/founder-cube-clean.png, public/supporters/founder-cube.png (+9 more)</t>
+        </is>
+      </c>
+      <c r="J130" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelog and excel report for commudle community integration
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>128 Commits Recorded</t>
+          <t>130 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>128 Actionable Milestones</t>
+          <t>130 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J130"/>
+  <dimension ref="A1:J132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7807,6 +7807,110 @@
         </is>
       </c>
       <c r="J130" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="40" customHeight="1">
+      <c r="A131" s="22" t="inlineStr">
+        <is>
+          <t>#130</t>
+        </is>
+      </c>
+      <c r="B131" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-02 20:49:09 +0530</t>
+        </is>
+      </c>
+      <c r="C131" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D131" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E131" s="23" t="inlineStr">
+        <is>
+          <t>4250f8e</t>
+        </is>
+      </c>
+      <c r="F131" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G131" s="24" t="inlineStr">
+        <is>
+          <t>docs: update changelog and excel report for supporter logos fix</t>
+        </is>
+      </c>
+      <c r="H131" s="24" t="inlineStr">
+        <is>
+          <t>docs: update changelog and excel report for supporter logos fix</t>
+        </is>
+      </c>
+      <c r="I131" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J131" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="40" customHeight="1">
+      <c r="A132" s="16" t="inlineStr">
+        <is>
+          <t>#131</t>
+        </is>
+      </c>
+      <c r="B132" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-02 21:19:37 +0530</t>
+        </is>
+      </c>
+      <c r="C132" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D132" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E132" s="17" t="inlineStr">
+        <is>
+          <t>2ba47d3</t>
+        </is>
+      </c>
+      <c r="F132" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G132" s="18" t="inlineStr">
+        <is>
+          <t>feat(community): link hero CTA and whats happening cards to official Commudle community and real workshop events</t>
+        </is>
+      </c>
+      <c r="H132" s="18" t="inlineStr">
+        <is>
+          <t>feat(community): link hero CTA and whats happening cards to official Commudle community and real workshop events</t>
+        </is>
+      </c>
+      <c r="I132" s="20" t="inlineStr">
+        <is>
+          <t>components/community/CommunityHero.tsx, components/community/WhatsHappeningSection.tsx, public/commudle-events/decode-the-machine.png, public/commudle-events/forging-the-ai-era.png, .../commudle-events/foundations-to-frontiers.png</t>
+        </is>
+      </c>
+      <c r="J132" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs: sync changelog and excel report for IST timezone fix
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>132 Commits Recorded</t>
+          <t>134 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>132 Actionable Milestones</t>
+          <t>134 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J134"/>
+  <dimension ref="A1:J136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8015,6 +8015,110 @@
         </is>
       </c>
       <c r="J134" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="40" customHeight="1">
+      <c r="A135" s="22" t="inlineStr">
+        <is>
+          <t>#134</t>
+        </is>
+      </c>
+      <c r="B135" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-02 21:50:29 +0530</t>
+        </is>
+      </c>
+      <c r="C135" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D135" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E135" s="23" t="inlineStr">
+        <is>
+          <t>29c04ba</t>
+        </is>
+      </c>
+      <c r="F135" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G135" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelog and excel report for automated event framework</t>
+        </is>
+      </c>
+      <c r="H135" s="24" t="inlineStr">
+        <is>
+          <t>docs: sync changelog and excel report for automated event framework</t>
+        </is>
+      </c>
+      <c r="I135" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J135" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="40" customHeight="1">
+      <c r="A136" s="16" t="inlineStr">
+        <is>
+          <t>#135</t>
+        </is>
+      </c>
+      <c r="B136" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-02 21:54:12 +0530</t>
+        </is>
+      </c>
+      <c r="C136" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D136" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E136" s="17" t="inlineStr">
+        <is>
+          <t>e1b4da6</t>
+        </is>
+      </c>
+      <c r="F136" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G136" s="18" t="inlineStr">
+        <is>
+          <t>fix(commudle): enforce Asia/Kolkata IST timezone for event start and end time formatting</t>
+        </is>
+      </c>
+      <c r="H136" s="18" t="inlineStr">
+        <is>
+          <t>fix(commudle): enforce Asia/Kolkata IST timezone for event start and end time formatting</t>
+        </is>
+      </c>
+      <c r="I136" s="20" t="inlineStr">
+        <is>
+          <t>lib/commudle.ts</t>
+        </is>
+      </c>
+      <c r="J136" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
fix(community): resolve event filtering for upcoming/past/all by latest date, add EventThumbnail direct unoptimized loading with fallback, and fix card opacity-0 re-render visibility
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>135 Commits Recorded</t>
+          <t>136 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>135 Actionable Milestones</t>
+          <t>136 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J137"/>
+  <dimension ref="A1:J138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8171,6 +8171,58 @@
         </is>
       </c>
       <c r="J137" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="40" customHeight="1">
+      <c r="A138" s="16" t="inlineStr">
+        <is>
+          <t>#137</t>
+        </is>
+      </c>
+      <c r="B138" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-02 22:00:57 +0530</t>
+        </is>
+      </c>
+      <c r="C138" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D138" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E138" s="17" t="inlineStr">
+        <is>
+          <t>c8b8fb6</t>
+        </is>
+      </c>
+      <c r="F138" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G138" s="18" t="inlineStr">
+        <is>
+          <t>docs: automated changelog and Excel report sync (iteration 26)</t>
+        </is>
+      </c>
+      <c r="H138" s="18" t="inlineStr">
+        <is>
+          <t>docs: automated changelog and Excel report sync (iteration 26)</t>
+        </is>
+      </c>
+      <c r="I138" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J138" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat(navbar): update navbar logo to official FORGE brand gear logo extracted from source document
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>136 Commits Recorded</t>
+          <t>137 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>136 Actionable Milestones</t>
+          <t>137 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J138"/>
+  <dimension ref="A1:J139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8223,6 +8223,58 @@
         </is>
       </c>
       <c r="J138" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="40" customHeight="1">
+      <c r="A139" s="22" t="inlineStr">
+        <is>
+          <t>#138</t>
+        </is>
+      </c>
+      <c r="B139" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-02 22:27:30 +0530</t>
+        </is>
+      </c>
+      <c r="C139" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D139" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E139" s="23" t="inlineStr">
+        <is>
+          <t>4a41d4d</t>
+        </is>
+      </c>
+      <c r="F139" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G139" s="24" t="inlineStr">
+        <is>
+          <t>fix(community): resolve event filtering for upcoming/past/all by latest date, add EventThumbnail direct unoptimized loading with fallback, and fix card opacity-0 re-render visibility</t>
+        </is>
+      </c>
+      <c r="H139" s="24" t="inlineStr">
+        <is>
+          <t>fix(community): resolve event filtering for upcoming/past/all by latest date, add EventThumbnail direct unoptimized loading with fallback, and fix card opacity-0 re-render visibility</t>
+        </is>
+      </c>
+      <c r="I139" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/community/WhatsHappeningSection.tsx</t>
+        </is>
+      </c>
+      <c r="J139" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat: incorporate 22 partner companies across collaborate and ecosystem pages
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>137 Commits Recorded</t>
+          <t>138 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>137 Actionable Milestones</t>
+          <t>138 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8275,6 +8275,58 @@
         </is>
       </c>
       <c r="J139" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="40" customHeight="1">
+      <c r="A140" s="16" t="inlineStr">
+        <is>
+          <t>#139</t>
+        </is>
+      </c>
+      <c r="B140" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-02 23:17:54 +0530</t>
+        </is>
+      </c>
+      <c r="C140" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D140" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E140" s="17" t="inlineStr">
+        <is>
+          <t>2cefdc4</t>
+        </is>
+      </c>
+      <c r="F140" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G140" s="18" t="inlineStr">
+        <is>
+          <t>feat(navbar): update navbar logo to official FORGE brand gear logo extracted from source document</t>
+        </is>
+      </c>
+      <c r="H140" s="18" t="inlineStr">
+        <is>
+          <t>feat(navbar): update navbar logo to official FORGE brand gear logo extracted from source document</t>
+        </is>
+      </c>
+      <c r="I140" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/Navbar.tsx (+6 more)</t>
+        </is>
+      </c>
+      <c r="J140" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
chore: update change reports for partner companies release
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>138 Commits Recorded</t>
+          <t>139 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>138 Actionable Milestones</t>
+          <t>139 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J140"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8327,6 +8327,58 @@
         </is>
       </c>
       <c r="J140" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="40" customHeight="1">
+      <c r="A141" s="22" t="inlineStr">
+        <is>
+          <t>#140</t>
+        </is>
+      </c>
+      <c r="B141" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-21 12:03:05 +0530</t>
+        </is>
+      </c>
+      <c r="C141" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D141" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E141" s="23" t="inlineStr">
+        <is>
+          <t>4f82bbc</t>
+        </is>
+      </c>
+      <c r="F141" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G141" s="24" t="inlineStr">
+        <is>
+          <t>feat: incorporate 22 partner companies across collaborate and ecosystem pages</t>
+        </is>
+      </c>
+      <c r="H141" s="24" t="inlineStr">
+        <is>
+          <t>feat: incorporate 22 partner companies across collaborate and ecosystem pages</t>
+        </is>
+      </c>
+      <c r="I141" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/collaborate/PartnerRepresentation.tsx (+24 more)</t>
+        </is>
+      </c>
+      <c r="J141" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat: regenerate all 22 partner logos in ultra-high resolution with 100% transparent backgrounds and replace legacy company logos across site
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>139 Commits Recorded</t>
+          <t>140 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>139 Actionable Milestones</t>
+          <t>140 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8379,6 +8379,58 @@
         </is>
       </c>
       <c r="J141" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="40" customHeight="1">
+      <c r="A142" s="16" t="inlineStr">
+        <is>
+          <t>#141</t>
+        </is>
+      </c>
+      <c r="B142" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-21 12:03:42 +0530</t>
+        </is>
+      </c>
+      <c r="C142" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D142" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E142" s="17" t="inlineStr">
+        <is>
+          <t>0e33bda</t>
+        </is>
+      </c>
+      <c r="F142" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G142" s="18" t="inlineStr">
+        <is>
+          <t>chore: update change reports for partner companies release</t>
+        </is>
+      </c>
+      <c r="H142" s="18" t="inlineStr">
+        <is>
+          <t>chore: update change reports for partner companies release</t>
+        </is>
+      </c>
+      <c r="I142" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J142" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
chore: update change reports for partner logos release
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>140 Commits Recorded</t>
+          <t>141 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>140 Actionable Milestones</t>
+          <t>141 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J142"/>
+  <dimension ref="A1:J143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8431,6 +8431,58 @@
         </is>
       </c>
       <c r="J142" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="40" customHeight="1">
+      <c r="A143" s="22" t="inlineStr">
+        <is>
+          <t>#142</t>
+        </is>
+      </c>
+      <c r="B143" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-21 13:17:22 +0530</t>
+        </is>
+      </c>
+      <c r="C143" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D143" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E143" s="23" t="inlineStr">
+        <is>
+          <t>d219bed</t>
+        </is>
+      </c>
+      <c r="F143" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G143" s="24" t="inlineStr">
+        <is>
+          <t>feat: regenerate all 22 partner logos in ultra-high resolution with 100% transparent backgrounds and replace legacy company logos across site</t>
+        </is>
+      </c>
+      <c r="H143" s="24" t="inlineStr">
+        <is>
+          <t>feat: regenerate all 22 partner logos in ultra-high resolution with 100% transparent backgrounds and replace legacy company logos across site</t>
+        </is>
+      </c>
+      <c r="I143" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/Hero.tsx (+32 more)</t>
+        </is>
+      </c>
+      <c r="J143" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat(hero): remove partners logos strip and fix landing page glitches
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>141 Commits Recorded</t>
+          <t>142 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>141 Actionable Milestones</t>
+          <t>142 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J143"/>
+  <dimension ref="A1:J144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8483,6 +8483,58 @@
         </is>
       </c>
       <c r="J143" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="40" customHeight="1">
+      <c r="A144" s="16" t="inlineStr">
+        <is>
+          <t>#143</t>
+        </is>
+      </c>
+      <c r="B144" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-21 13:18:17 +0530</t>
+        </is>
+      </c>
+      <c r="C144" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D144" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E144" s="17" t="inlineStr">
+        <is>
+          <t>22f653e</t>
+        </is>
+      </c>
+      <c r="F144" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G144" s="18" t="inlineStr">
+        <is>
+          <t>chore: update change reports for partner logos release</t>
+        </is>
+      </c>
+      <c r="H144" s="18" t="inlineStr">
+        <is>
+          <t>chore: update change reports for partner logos release</t>
+        </is>
+      </c>
+      <c r="I144" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J144" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
fix(landing): remove unnecessary buttons and fix layout glitches
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>142 Commits Recorded</t>
+          <t>143 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>142 Actionable Milestones</t>
+          <t>143 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J144"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8535,6 +8535,58 @@
         </is>
       </c>
       <c r="J144" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="40" customHeight="1">
+      <c r="A145" s="22" t="inlineStr">
+        <is>
+          <t>#144</t>
+        </is>
+      </c>
+      <c r="B145" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:22:07 +0530</t>
+        </is>
+      </c>
+      <c r="C145" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D145" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E145" s="23" t="inlineStr">
+        <is>
+          <t>9f0a69b</t>
+        </is>
+      </c>
+      <c r="F145" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G145" s="24" t="inlineStr">
+        <is>
+          <t>feat(hero): remove partners logos strip and fix landing page glitches</t>
+        </is>
+      </c>
+      <c r="H145" s="24" t="inlineStr">
+        <is>
+          <t>feat(hero): remove partners logos strip and fix landing page glitches</t>
+        </is>
+      </c>
+      <c r="I145" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_ANIMATION_CATALOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt (+6 more)</t>
+        </is>
+      </c>
+      <c r="J145" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat(courses): integrate 26 course brochures across 1-year, 6-months, 3-months, and 45-days durations with catalog and download flows
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>143 Commits Recorded</t>
+          <t>144 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>143 Actionable Milestones</t>
+          <t>144 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J145"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8587,6 +8587,58 @@
         </is>
       </c>
       <c r="J145" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="40" customHeight="1">
+      <c r="A146" s="16" t="inlineStr">
+        <is>
+          <t>#145</t>
+        </is>
+      </c>
+      <c r="B146" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:37:11 +0530</t>
+        </is>
+      </c>
+      <c r="C146" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D146" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E146" s="17" t="inlineStr">
+        <is>
+          <t>d7fe88f</t>
+        </is>
+      </c>
+      <c r="F146" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G146" s="18" t="inlineStr">
+        <is>
+          <t>fix(landing): remove unnecessary buttons and fix layout glitches</t>
+        </is>
+      </c>
+      <c r="H146" s="18" t="inlineStr">
+        <is>
+          <t>fix(landing): remove unnecessary buttons and fix layout glitches</t>
+        </is>
+      </c>
+      <c r="I146" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/Hero.tsx (+7 more)</t>
+        </is>
+      </c>
+      <c r="J146" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat(courses): redesign Courses by Duration with editorial hero, 2D vector illustrations, dynamic duration tabs, and 6-card initial view
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>144 Commits Recorded</t>
+          <t>145 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>144 Actionable Milestones</t>
+          <t>145 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8639,6 +8639,58 @@
         </is>
       </c>
       <c r="J146" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="40" customHeight="1">
+      <c r="A147" s="22" t="inlineStr">
+        <is>
+          <t>#146</t>
+        </is>
+      </c>
+      <c r="B147" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:26:56 +0530</t>
+        </is>
+      </c>
+      <c r="C147" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D147" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E147" s="23" t="inlineStr">
+        <is>
+          <t>8a74d44</t>
+        </is>
+      </c>
+      <c r="F147" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G147" s="24" t="inlineStr">
+        <is>
+          <t>feat(courses): integrate 26 course brochures across 1-year, 6-months, 3-months, and 45-days durations with catalog and download flows</t>
+        </is>
+      </c>
+      <c r="H147" s="24" t="inlineStr">
+        <is>
+          <t>feat(courses): integrate 26 course brochures across 1-year, 6-months, 3-months, and 45-days durations with catalog and download flows</t>
+        </is>
+      </c>
+      <c r="I147" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, app/courses/page.tsx, changes.txt (+37 more)</t>
+        </is>
+      </c>
+      <c r="J147" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs(changelog): update reports for courses section redesign
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>145 Commits Recorded</t>
+          <t>146 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>145 Actionable Milestones</t>
+          <t>146 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J147"/>
+  <dimension ref="A1:J148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8691,6 +8691,58 @@
         </is>
       </c>
       <c r="J147" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="40" customHeight="1">
+      <c r="A148" s="16" t="inlineStr">
+        <is>
+          <t>#147</t>
+        </is>
+      </c>
+      <c r="B148" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:11:11 +0530</t>
+        </is>
+      </c>
+      <c r="C148" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D148" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E148" s="17" t="inlineStr">
+        <is>
+          <t>39ec414</t>
+        </is>
+      </c>
+      <c r="F148" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G148" s="18" t="inlineStr">
+        <is>
+          <t>feat(courses): redesign Courses by Duration with editorial hero, 2D vector illustrations, dynamic duration tabs, and 6-card initial view</t>
+        </is>
+      </c>
+      <c r="H148" s="18" t="inlineStr">
+        <is>
+          <t>feat(courses): redesign Courses by Duration with editorial hero, 2D vector illustrations, dynamic duration tabs, and 6-card initial view</t>
+        </is>
+      </c>
+      <c r="I148" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/programs/CourseCatalogSection.tsx (+29 more)</t>
+        </is>
+      </c>
+      <c r="J148" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat(courses): replace vector illustrations with high-res authentic real photography across course catalog cards and hero
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>146 Commits Recorded</t>
+          <t>147 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>146 Actionable Milestones</t>
+          <t>147 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J148"/>
+  <dimension ref="A1:J149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8743,6 +8743,58 @@
         </is>
       </c>
       <c r="J148" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="40" customHeight="1">
+      <c r="A149" s="22" t="inlineStr">
+        <is>
+          <t>#148</t>
+        </is>
+      </c>
+      <c r="B149" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:12:27 +0530</t>
+        </is>
+      </c>
+      <c r="C149" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D149" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E149" s="23" t="inlineStr">
+        <is>
+          <t>39b8959</t>
+        </is>
+      </c>
+      <c r="F149" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G149" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update reports for courses section redesign</t>
+        </is>
+      </c>
+      <c r="H149" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update reports for courses section redesign</t>
+        </is>
+      </c>
+      <c r="I149" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J149" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs(changelog): update change report for real course images
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>147 Commits Recorded</t>
+          <t>148 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>147 Actionable Milestones</t>
+          <t>148 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J149"/>
+  <dimension ref="A1:J150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8795,6 +8795,58 @@
         </is>
       </c>
       <c r="J149" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="40" customHeight="1">
+      <c r="A150" s="16" t="inlineStr">
+        <is>
+          <t>#149</t>
+        </is>
+      </c>
+      <c r="B150" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:40:30 +0530</t>
+        </is>
+      </c>
+      <c r="C150" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D150" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E150" s="17" t="inlineStr">
+        <is>
+          <t>44f5830</t>
+        </is>
+      </c>
+      <c r="F150" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G150" s="18" t="inlineStr">
+        <is>
+          <t>feat(courses): replace vector illustrations with high-res authentic real photography across course catalog cards and hero</t>
+        </is>
+      </c>
+      <c r="H150" s="18" t="inlineStr">
+        <is>
+          <t>feat(courses): replace vector illustrations with high-res authentic real photography across course catalog cards and hero</t>
+        </is>
+      </c>
+      <c r="I150" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/programs/CourseCatalogSection.tsx (+10 more)</t>
+        </is>
+      </c>
+      <c r="J150" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
feat(courses): gate brochure downloads and PDF previews with student details form and interactive mobile OTP verification
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>148 Commits Recorded</t>
+          <t>149 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>148 Actionable Milestones</t>
+          <t>149 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8847,6 +8847,58 @@
         </is>
       </c>
       <c r="J150" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="40" customHeight="1">
+      <c r="A151" s="22" t="inlineStr">
+        <is>
+          <t>#150</t>
+        </is>
+      </c>
+      <c r="B151" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:40:47 +0530</t>
+        </is>
+      </c>
+      <c r="C151" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D151" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E151" s="23" t="inlineStr">
+        <is>
+          <t>eaa11f4</t>
+        </is>
+      </c>
+      <c r="F151" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G151" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update change report for real course images</t>
+        </is>
+      </c>
+      <c r="H151" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update change report for real course images</t>
+        </is>
+      </c>
+      <c r="I151" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J151" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs(changelog): update reports for OTP brochure flow
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>149 Commits Recorded</t>
+          <t>150 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>149 Actionable Milestones</t>
+          <t>150 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8899,6 +8899,58 @@
         </is>
       </c>
       <c r="J151" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="40" customHeight="1">
+      <c r="A152" s="16" t="inlineStr">
+        <is>
+          <t>#151</t>
+        </is>
+      </c>
+      <c r="B152" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:23:54 +0530</t>
+        </is>
+      </c>
+      <c r="C152" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D152" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E152" s="17" t="inlineStr">
+        <is>
+          <t>aa969c1</t>
+        </is>
+      </c>
+      <c r="F152" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G152" s="18" t="inlineStr">
+        <is>
+          <t>feat(courses): gate brochure downloads and PDF previews with student details form and interactive mobile OTP verification</t>
+        </is>
+      </c>
+      <c r="H152" s="18" t="inlineStr">
+        <is>
+          <t>feat(courses): gate brochure downloads and PDF previews with student details form and interactive mobile OTP verification</t>
+        </is>
+      </c>
+      <c r="I152" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/modal/DownloadForm.tsx (+3 more)</t>
+        </is>
+      </c>
+      <c r="J152" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
refactor(courses): remove OTP verification and restore direct download and preview links
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>150 Commits Recorded</t>
+          <t>151 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>150 Actionable Milestones</t>
+          <t>151 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J152"/>
+  <dimension ref="A1:J153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8951,6 +8951,58 @@
         </is>
       </c>
       <c r="J152" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="40" customHeight="1">
+      <c r="A153" s="22" t="inlineStr">
+        <is>
+          <t>#152</t>
+        </is>
+      </c>
+      <c r="B153" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:24:04 +0530</t>
+        </is>
+      </c>
+      <c r="C153" s="24" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D153" s="22" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E153" s="23" t="inlineStr">
+        <is>
+          <t>56e7980</t>
+        </is>
+      </c>
+      <c r="F153" s="25" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G153" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update reports for OTP brochure flow</t>
+        </is>
+      </c>
+      <c r="H153" s="24" t="inlineStr">
+        <is>
+          <t>docs(changelog): update reports for OTP brochure flow</t>
+        </is>
+      </c>
+      <c r="I153" s="26" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt</t>
+        </is>
+      </c>
+      <c r="J153" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>

<commit_message>
docs(changelog): update reports after removing OTP
</commit_message>
<xml_diff>
--- a/FORGE_Website_Project_Change_Report.xlsx
+++ b/FORGE_Website_Project_Change_Report.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>151 Commits Recorded</t>
+          <t>152 Commits Recorded</t>
         </is>
       </c>
       <c r="C7" s="27" t="n"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>151 Actionable Milestones</t>
+          <t>152 Actionable Milestones</t>
         </is>
       </c>
       <c r="C8" s="27" t="n"/>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9003,6 +9003,58 @@
         </is>
       </c>
       <c r="J153" s="21" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="40" customHeight="1">
+      <c r="A154" s="16" t="inlineStr">
+        <is>
+          <t>#153</t>
+        </is>
+      </c>
+      <c r="B154" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:32:55 +0530</t>
+        </is>
+      </c>
+      <c r="C154" s="18" t="inlineStr">
+        <is>
+          <t>Continuous Updates</t>
+        </is>
+      </c>
+      <c r="D154" s="16" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="E154" s="17" t="inlineStr">
+        <is>
+          <t>b08838f</t>
+        </is>
+      </c>
+      <c r="F154" s="19" t="inlineStr">
+        <is>
+          <t>Winnovation</t>
+        </is>
+      </c>
+      <c r="G154" s="18" t="inlineStr">
+        <is>
+          <t>refactor(courses): remove OTP verification and restore direct download and preview links</t>
+        </is>
+      </c>
+      <c r="H154" s="18" t="inlineStr">
+        <is>
+          <t>refactor(courses): remove OTP verification and restore direct download and preview links</t>
+        </is>
+      </c>
+      <c r="I154" s="20" t="inlineStr">
+        <is>
+          <t>CHANGES_LOG.txt, FORGE_Website_Project_Change_Report.csv, FORGE_Website_Project_Change_Report.xlsx, changes.txt, components/modal/DownloadForm.tsx (+2 more)</t>
+        </is>
+      </c>
+      <c r="J154" s="21" t="inlineStr">
         <is>
           <t>Committed</t>
         </is>

</xml_diff>